<commit_message>
Add runtime graph dataset v2 workers=40, 10-6k records
</commit_message>
<xml_diff>
--- a/reports/runtimes.xlsx
+++ b/reports/runtimes.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/codeathon2026/metadata-curation-harmonization/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB91C2D4-18F4-E343-8512-7C7CBA1AE4BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11785194-BEDF-7449-931A-C98BB59A7624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4060" yWindow="2580" windowWidth="27240" windowHeight="16180" activeTab="1" xr2:uid="{39223533-88C1-324C-BCB7-CCCCEFC6E7F0}"/>
+    <workbookView xWindow="4060" yWindow="2580" windowWidth="27240" windowHeight="16180" activeTab="2" xr2:uid="{39223533-88C1-324C-BCB7-CCCCEFC6E7F0}"/>
   </bookViews>
   <sheets>
     <sheet name="v1.curated.309uniq" sheetId="2" r:id="rId1"/>
     <sheet name="v1.data" sheetId="1" r:id="rId2"/>
+    <sheet name="v2.records_vs_time" sheetId="4" r:id="rId3"/>
+    <sheet name="v2.data" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="38">
   <si>
     <t>Machine</t>
   </si>
@@ -133,6 +135,27 @@
   </si>
   <si>
     <t>     232 dataset/v2/curated_combined.unique_isolation_host.jsonl</t>
+  </si>
+  <si>
+    <t>V2</t>
+  </si>
+  <si>
+    <t>0m20s</t>
+  </si>
+  <si>
+    <t>232_unique</t>
+  </si>
+  <si>
+    <t>6k_curated</t>
+  </si>
+  <si>
+    <t>13m27s</t>
+  </si>
+  <si>
+    <t>168k_combined</t>
+  </si>
+  <si>
+    <t>Records</t>
   </si>
 </sst>
 </file>
@@ -260,7 +283,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -280,18 +303,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -306,6 +317,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -998,7 +1030,570 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="3200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="3200"/>
+              <a:t>dataset</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="3200" baseline="0"/>
+              <a:t> v2; workers =40, records vs time</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="3200"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="3200" baseline="0"/>
+              <a:t>Macbook Pro M4 48G RAM 14 cores</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="3200"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="3200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'v2.data'!$G$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Seconds</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="101600">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="r"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'v2.data'!$F$13:$F$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>232</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>168000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'v2.data'!$G$13:$G$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>87</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-85CF-374A-818E-E6D9A72E703A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="638207295"/>
+        <c:axId val="526049599"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="638207295"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="10000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800"/>
+                  <a:t>records</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="526049599"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="526049599"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800"/>
+                  <a:t>runtime in seconds</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="638207295"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1554,8 +2149,532 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{FD96F575-9D82-314D-8471-6CB914880F52}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{7420B6BE-29B8-D043-BA7D-899878F36EC6}">
   <sheetPr/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1573,6 +2692,39 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC2887AB-E3DE-CB7D-C5A6-C1B1D5613BE7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="8662051" cy="6274017"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD984D67-349C-F86B-5656-C2DF1F7E28F2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2019,10 +3171,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="9">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="14">
         <v>50</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -2034,10 +3186,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="10"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="15"/>
       <c r="E8" s="5" t="s">
         <v>14</v>
       </c>
@@ -2094,66 +3246,66 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="7" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="8" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
+      <c r="A16" s="8"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="10" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="15"/>
+      <c r="A21" s="11"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11"/>
+      <c r="A22" s="7"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="10" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="10" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
+      <c r="A27" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2168,4 +3320,341 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28738C45-BFFF-294C-921D-53562624ABDF}">
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+    </row>
+    <row r="2" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="17"/>
+      <c r="G2">
+        <f>INT(LEFT(E2,1))*60+INT(LEFT(RIGHT(E2,3),2))</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="18"/>
+      <c r="G3">
+        <f>INT(LEFT(E3,1))*60+INT(LEFT(RIGHT(E3,3),2))</f>
+        <v>170</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="17"/>
+      <c r="G4">
+        <f t="shared" ref="G4:G11" si="0">INT(LEFT(E4,1))*60+INT(LEFT(RIGHT(E4,3),2))</f>
+        <v>134</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2">
+        <v>30</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="17"/>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>80</v>
+      </c>
+      <c r="J5" s="8"/>
+    </row>
+    <row r="6" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2">
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="17"/>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="12"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="14">
+        <v>50</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="18"/>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>68</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="18"/>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>57</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="3">
+        <v>100</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="18"/>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>71</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="3">
+        <v>400</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="18"/>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>104</v>
+      </c>
+      <c r="J10" s="11"/>
+    </row>
+    <row r="11" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="2">
+        <v>10</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="17"/>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>248</v>
+      </c>
+      <c r="J11" s="7"/>
+    </row>
+    <row r="12" spans="1:10" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="2">
+        <v>30</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="17">
+        <v>10</v>
+      </c>
+      <c r="G13">
+        <f>INT(LEFT(E13,1))*60+INT(LEFT(RIGHT(E13,3),2))</f>
+        <v>20</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="2">
+        <v>40</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="17">
+        <v>232</v>
+      </c>
+      <c r="G14">
+        <f>INT(LEFT(E14,1))*60+INT(LEFT(RIGHT(E14,3),2))</f>
+        <v>65</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="2">
+        <v>40</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="18">
+        <v>6000</v>
+      </c>
+      <c r="G15">
+        <f t="shared" ref="G15:G16" si="1">INT(LEFT(E15,1))*60+INT(LEFT(RIGHT(E15,3),2))</f>
+        <v>87</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="2">
+        <v>40</v>
+      </c>
+      <c r="E16" s="3"/>
+      <c r="F16" s="18">
+        <v>168000</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="J6" r:id="rId1" display="https://ftp.ncbi.nlm.nih.gov/.baby/datafiles/.argonne/combined.jsonl.gz" xr:uid="{B15C7EA7-293C-0A4A-A283-EFA8D469566C}"/>
+    <hyperlink ref="J12" r:id="rId2" display="https://ftp.ncbi.nlm.nih.gov/pub/datasets/.argonne/combined.v2.jsonl.gz" xr:uid="{ADB35956-D29D-4D4D-9F29-A848CD5CA303}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add daytime 40 worker 10,232,6000 runtimes, v2 data, openminded planner code
</commit_message>
<xml_diff>
--- a/reports/runtimes.xlsx
+++ b/reports/runtimes.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/codeathon2026/metadata-curation-harmonization/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86722E19-0897-5D42-A6AC-C7AE69C05822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4735B25-1529-3D42-A605-E76196817CE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4060" yWindow="2580" windowWidth="27240" windowHeight="16180" activeTab="3" xr2:uid="{39223533-88C1-324C-BCB7-CCCCEFC6E7F0}"/>
+    <workbookView xWindow="4060" yWindow="2580" windowWidth="27240" windowHeight="16180" activeTab="4" xr2:uid="{39223533-88C1-324C-BCB7-CCCCEFC6E7F0}"/>
   </bookViews>
   <sheets>
     <sheet name="v1.curated.309uniq" sheetId="2" r:id="rId1"/>
     <sheet name="v1.data" sheetId="1" r:id="rId2"/>
     <sheet name="v2.records_vs_time" sheetId="4" r:id="rId3"/>
     <sheet name="v2.data" sheetId="3" r:id="rId4"/>
+    <sheet name="v2.openminded.chart" sheetId="6" r:id="rId5"/>
+    <sheet name="v2.openmined.data" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="45">
   <si>
     <t>Machine</t>
   </si>
@@ -157,12 +159,33 @@
   <si>
     <t>Records</t>
   </si>
+  <si>
+    <t>command</t>
+  </si>
+  <si>
+    <t>conda run -n orchestrator --no-capture-output python3 scripts/run_pipeline.py  --log-level DEBUG  --set workers=40 --set records=dataset/v2/curated_combined.head10.jsonl --run v2head10-openminded</t>
+  </si>
+  <si>
+    <t>uniq</t>
+  </si>
+  <si>
+    <t>conda run -n orchestrator --no-capture-output python3 scripts/run_pipeline.py  --log-level DEBUG  --set workers=40 --set records=dataset/v2/curated_combined.unique_isolation_host.jsonl  --run v2uniq-openminded</t>
+  </si>
+  <si>
+    <t>Curated</t>
+  </si>
+  <si>
+    <t>conda run -n orchestrator --no-capture-output python3 scripts/run_pipeline.py  --log-level DEBUG  --set workers=40 --set records=dataset/v2/curated_combined.jsonl  --run v2curated-openminded</t>
+  </si>
+  <si>
+    <t>records</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -208,6 +231,26 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8.25"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8.25"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -283,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -318,6 +361,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -330,15 +382,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1553,6 +1612,543 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800"/>
+              <a:t>v2 dataset</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1800" baseline="0"/>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1800" baseline="0"/>
+              <a:t>using "openminded" planning agent, 40 workers</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1800"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'v2.openmined.data'!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Time</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="127000">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.4661654612747026E-3"/>
+                  <c:y val="-4.6557094123270776E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:separator>; </c:separator>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-66F9-3C46-9D4C-5F888FE7ED1D}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1600" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:separator>; </c:separator>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'v2.openmined.data'!$E$2:$E$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>232</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'v2.openmined.data'!$F$2:$F$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>29.106999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>75.599999999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1095.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-66F9-3C46-9D4C-5F888FE7ED1D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="755502143"/>
+        <c:axId val="755500351"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="755502143"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800"/>
+                  <a:t>Records</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="755500351"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="755500351"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800"/>
+                  <a:t>Runtime in seconds</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="755502143"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1633,6 +2229,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2150,6 +2786,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2675,6 +3827,14 @@
 
 <file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{7420B6BE-29B8-D043-BA7D-899878F36EC6}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/chartsheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{48BA8F4D-5D52-254F-AA10-BAFC5570AAD3}">
   <sheetPr/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2718,13 +3878,46 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="8662051" cy="6284872"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD984D67-349C-F86B-5656-C2DF1F7E28F2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
     <xdr:ext cx="8662051" cy="6274017"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CD984D67-349C-F86B-5656-C2DF1F7E28F2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C74B217F-EDE9-3A4B-CD08-43C0B3909D74}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3171,10 +4364,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="14">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
         <v>50</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -3186,10 +4379,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="15"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="5" t="s">
         <v>14</v>
       </c>
@@ -3347,8 +4540,8 @@
       <c r="G1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:10" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -3366,7 +4559,7 @@
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="17"/>
+      <c r="F2" s="13"/>
       <c r="G2">
         <f>INT(LEFT(E2,1))*60+INT(LEFT(RIGHT(E2,3),2))</f>
         <v>28</v>
@@ -3384,7 +4577,7 @@
       <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="18"/>
+      <c r="F3" s="14"/>
       <c r="G3">
         <f>INT(LEFT(E3,1))*60+INT(LEFT(RIGHT(E3,3),2))</f>
         <v>170</v>
@@ -3403,7 +4596,7 @@
       <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="17"/>
+      <c r="F4" s="13"/>
       <c r="G4">
         <f t="shared" ref="G4:G11" si="0">INT(LEFT(E4,1))*60+INT(LEFT(RIGHT(E4,3),2))</f>
         <v>134</v>
@@ -3422,7 +4615,7 @@
       <c r="E5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="17"/>
+      <c r="F5" s="13"/>
       <c r="G5">
         <f t="shared" si="0"/>
         <v>80</v>
@@ -3439,7 +4632,7 @@
       <c r="E6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="17"/>
+      <c r="F6" s="13"/>
       <c r="G6">
         <f t="shared" si="0"/>
         <v>65</v>
@@ -3449,16 +4642,16 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="14">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="17">
         <v>50</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="18"/>
+      <c r="F7" s="14"/>
       <c r="G7">
         <f t="shared" si="0"/>
         <v>68</v>
@@ -3468,14 +4661,14 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="15"/>
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="18"/>
       <c r="E8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="18"/>
+      <c r="F8" s="14"/>
       <c r="G8">
         <f t="shared" si="0"/>
         <v>57</v>
@@ -3494,7 +4687,7 @@
       <c r="E9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F9" s="18"/>
+      <c r="F9" s="14"/>
       <c r="G9">
         <f t="shared" si="0"/>
         <v>71</v>
@@ -3513,7 +4706,7 @@
       <c r="E10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="18"/>
+      <c r="F10" s="14"/>
       <c r="G10">
         <f t="shared" si="0"/>
         <v>104</v>
@@ -3532,7 +4725,7 @@
       <c r="E11" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="17"/>
+      <c r="F11" s="13"/>
       <c r="G11">
         <f t="shared" si="0"/>
         <v>248</v>
@@ -3551,8 +4744,8 @@
       <c r="G12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H12" s="16"/>
-      <c r="I12" s="16"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
       <c r="J12" s="9" t="s">
         <v>27</v>
       </c>
@@ -3573,7 +4766,7 @@
       <c r="E13" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="13">
         <v>10</v>
       </c>
       <c r="G13">
@@ -3596,7 +4789,7 @@
       <c r="E14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="17">
+      <c r="F14" s="13">
         <v>232</v>
       </c>
       <c r="G14">
@@ -3619,11 +4812,11 @@
       <c r="E15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="18">
+      <c r="F15" s="14">
         <v>6000</v>
       </c>
       <c r="G15">
-        <f t="shared" ref="G15:G16" si="1">INT(LEFT(E15,1))*60+INT(LEFT(RIGHT(E15,3),2))</f>
+        <f t="shared" ref="G15" si="1">INT(LEFT(E15,1))*60+INT(LEFT(RIGHT(E15,3),2))</f>
         <v>87</v>
       </c>
       <c r="J15" s="10" t="s">
@@ -3640,7 +4833,7 @@
         <v>40</v>
       </c>
       <c r="E16" s="3"/>
-      <c r="F16" s="18">
+      <c r="F16" s="14">
         <v>168000</v>
       </c>
     </row>
@@ -3657,4 +4850,101 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8D69E7-657E-D045-ACA6-B29262624136}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="7" max="7" width="10.83203125" style="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="45" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="19">
+        <v>40</v>
+      </c>
+      <c r="E2" s="19">
+        <v>10</v>
+      </c>
+      <c r="F2" s="19">
+        <v>29.106999999999999</v>
+      </c>
+      <c r="G2" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="2">
+        <v>40</v>
+      </c>
+      <c r="E3" s="2">
+        <v>232</v>
+      </c>
+      <c r="F3" s="20">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="2">
+        <v>40</v>
+      </c>
+      <c r="E4" s="2">
+        <v>6000</v>
+      </c>
+      <c r="F4" s="20">
+        <v>1095.3</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>